<commit_message>
v0.7 accepted + folded into architecture.md; DNL B17 annotated; engine plan
- architecture.md -> v0.7 with v0.6->v0.7 migration note (six process-discipline
  refinements: 3.7, 16.5, 11.6, 4.4.1, 3.5.7, 14.5.2). Proposal marked ACCEPTED.
- lint backported: DNL v6 + WBC v4 both lint-clean (exit 0)
- DNL B17 'DM real GDP growth' annotated as context memo -> lint WARN not ERROR; no value change
- design/engine_implementation_plan.md: steps 6+10 plan (linkage/assumptions, fcf/bank
  engines, golden-master tests, M0-M5, R1-R8) FOR APPROVAL
- WORKING_NOTES handoff updated
</commit_message>
<xml_diff>
--- a/analyses/dnl/valuations/dnl_muddle_through_valuation_v6_2026-06-25.xlsx
+++ b/analyses/dnl/valuations/dnl_muddle_through_valuation_v6_2026-06-25.xlsx
@@ -2100,7 +2100,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="19.5" customHeight="1" s="67">
       <c r="A8" s="75" t="inlineStr">
         <is>
@@ -2231,7 +2230,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="19.5" customHeight="1" s="67">
       <c r="A16" s="75" t="inlineStr">
         <is>
@@ -2245,7 +2243,7 @@
     <row r="17" ht="15" customHeight="1" s="67">
       <c r="A17" s="71" t="inlineStr">
         <is>
-          <t>DM real GDP growth</t>
+          <t>DM real GDP growth (context memo)</t>
         </is>
       </c>
       <c r="B17" s="155" t="n">
@@ -2253,7 +2251,7 @@
       </c>
       <c r="C17" s="78" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>Macro-baseline context only — NOT used in the growth chain, which keys off global mining real growth (B19) and inflation (B18). Shown for reference. [context memo]</t>
         </is>
       </c>
       <c r="D17" s="71" t="inlineStr">
@@ -2322,7 +2320,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="19.5" customHeight="1" s="67">
       <c r="A22" s="75" t="inlineStr">
         <is>
@@ -2480,7 +2477,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32" ht="19.5" customHeight="1" s="67">
       <c r="A32" s="75" t="inlineStr">
         <is>
@@ -2686,7 +2682,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
     <row r="44" ht="19.5" customHeight="1" s="67">
       <c r="A44" s="75" t="inlineStr">
         <is>
@@ -2797,7 +2792,6 @@
         </is>
       </c>
     </row>
-    <row r="50"/>
     <row r="51" ht="19.5" customHeight="1" s="67">
       <c r="A51" s="75" t="inlineStr">
         <is>
@@ -2908,7 +2902,6 @@
         </is>
       </c>
     </row>
-    <row r="57"/>
     <row r="58" ht="19.5" customHeight="1" s="67">
       <c r="A58" s="75" t="inlineStr">
         <is>
@@ -3077,7 +3070,6 @@
         </is>
       </c>
     </row>
-    <row r="67"/>
     <row r="68" ht="19.5" customHeight="1" s="67">
       <c r="A68" s="75" t="inlineStr">
         <is>
@@ -3204,7 +3196,6 @@
         </is>
       </c>
     </row>
-    <row r="75"/>
     <row r="76" ht="19.5" customHeight="1" s="67">
       <c r="A76" s="75" t="inlineStr">
         <is>
@@ -3255,7 +3246,6 @@
         </is>
       </c>
     </row>
-    <row r="79"/>
     <row r="80" ht="19.5" customHeight="1" s="67">
       <c r="A80" s="75" t="inlineStr">
         <is>
@@ -3286,7 +3276,6 @@
         </is>
       </c>
     </row>
-    <row r="82"/>
     <row r="83" ht="19.5" customHeight="1" s="67">
       <c r="A83" s="75" t="inlineStr">
         <is>
@@ -3378,7 +3367,6 @@
         </is>
       </c>
     </row>
-    <row r="88"/>
     <row r="89" ht="19.5" customHeight="1" s="67">
       <c r="A89" s="75" t="inlineStr">
         <is>
@@ -3753,7 +3741,6 @@
         </is>
       </c>
     </row>
-    <row r="108"/>
     <row r="109" ht="19.5" customHeight="1" s="67">
       <c r="A109" s="75" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
DNL lease accounting (Approach A re-anchor: MT 3.48, materiality panel, lint lease-basis check, data-contract stub) + prior UI build-out (beta determinants, summary financials, multiples tab + peer workbench, DCF table)
</commit_message>
<xml_diff>
--- a/analyses/dnl/valuations/dnl_muddle_through_valuation_v6_2026-06-25.xlsx
+++ b/analyses/dnl/valuations/dnl_muddle_through_valuation_v6_2026-06-25.xlsx
@@ -1363,7 +1363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="50" customWidth="1" style="66" min="1" max="1"/>
@@ -1707,67 +1707,79 @@
       </c>
     </row>
     <row r="30" ht="17.35" customHeight="1" s="67">
-      <c r="A30" s="143" t="inlineStr">
+      <c r="A30" s="66" t="inlineStr">
+        <is>
+          <t>Less: AASB 16 lease liabilities (Approach A: leases = debt)</t>
+        </is>
+      </c>
+      <c r="C30" s="66">
+        <f>-Assumptions!$B$108</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="67">
+      <c r="A31" s="143" t="inlineStr">
         <is>
           <t>Equity value</t>
         </is>
       </c>
-      <c r="C30" s="146">
-        <f>C27+C28+C29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="15" customHeight="1" s="67">
-      <c r="A31" s="96" t="inlineStr">
+      <c r="C31" s="146">
+        <f>C27+C28+C29+C30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="19.7" customHeight="1" s="67">
+      <c r="A32" s="96" t="inlineStr">
         <is>
           <t>Divided by shares outstanding (Q8: H1 anchor, no buyback projection)</t>
         </is>
       </c>
-      <c r="C31" s="103">
+      <c r="C32" s="103">
         <f>Assumptions!$B$81</f>
         <v/>
       </c>
     </row>
-    <row r="32" ht="19.7" customHeight="1" s="67">
-      <c r="A32" s="147" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="147" t="inlineStr">
         <is>
           <t>VALUE PER SHARE</t>
         </is>
       </c>
-      <c r="C32" s="148">
-        <f>C30/C31</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" ht="21.75" customHeight="1" s="67">
-      <c r="A34" s="75" t="inlineStr">
+      <c r="C33" s="148">
+        <f>C31/C32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="21.75" customHeight="1" s="67"/>
+    <row r="35" ht="15" customHeight="1" s="67">
+      <c r="A35" s="75" t="inlineStr">
         <is>
           <t>MARKET CHECK</t>
         </is>
       </c>
-      <c r="B34" s="76" t="n"/>
-      <c r="C34" s="76" t="n"/>
-      <c r="D34" s="76" t="n"/>
-    </row>
-    <row r="35" ht="15" customHeight="1" s="67">
-      <c r="A35" s="96" t="inlineStr">
-        <is>
-          <t>Market reference per share</t>
-        </is>
-      </c>
-      <c r="C35" s="149">
-        <f>Assumptions!$B$110</f>
-        <v/>
-      </c>
+      <c r="B35" s="76" t="n"/>
+      <c r="C35" s="76" t="n"/>
+      <c r="D35" s="76" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1" s="67">
       <c r="A36" s="96" t="inlineStr">
         <is>
+          <t>Market reference per share</t>
+        </is>
+      </c>
+      <c r="C36" s="149">
+        <f>Assumptions!$B$110</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="96" t="inlineStr">
+        <is>
           <t>Discount / (premium) vs market</t>
         </is>
       </c>
-      <c r="C36" s="106">
-        <f>C32/C35-1</f>
+      <c r="C37" s="106">
+        <f>C33/C36-1</f>
         <v/>
       </c>
     </row>
@@ -3738,6 +3750,21 @@
       <c r="D107" s="71" t="inlineStr">
         <is>
           <t>Face x probability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="66" t="inlineStr">
+        <is>
+          <t>AASB 16 lease liabilities (H1 val date)</t>
+        </is>
+      </c>
+      <c r="B108" s="66" t="n">
+        <v>194.3</v>
+      </c>
+      <c r="D108" s="66" t="inlineStr">
+        <is>
+          <t>H1 FY26 balance sheet (matches Balance Sheet lease liabilities). Added explicitly to the equity bridge per Approach A (leases treated as debt); reported net debt is ex-leases.</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4678,7 @@
       </c>
       <c r="C20" s="71" t="inlineStr">
         <is>
-          <t>Interest-bearing liabilities + capital leases - cash - hedging derivatives. Up AUD 80m H/H: buyback AUD 128m + dividends paid AUD 170m - Gibson Island proceeds AUD 198m.</t>
+          <t>Interest-bearing borrowings less cash and hedging derivatives. AASB 16 lease liabilities (shown separately above) are NOT included here; they are deducted explicitly in the equity bridge per Approach A. Up AUD 80m H/H.</t>
         </is>
       </c>
     </row>

</xml_diff>